<commit_message>
rebuild the geopackage, derive watersheds with FWAPGR, add geopackage with new stream locations.
</commit_message>
<xml_diff>
--- a/data/habitat_confirmations_priorities.xlsx
+++ b/data/habitat_confirmations_priorities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\OneDrive\New_Graph\Current\2020-025_cwf_elk\scripts\fish_passage_elk_2020_reporting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42FA5414-211E-4B97-A554-83887E4C9F69}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46A152F-750A-41EB-9C6C-5C013CD1F34C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{821C12C4-A1B8-974C-A56E-63CAEF8E23F0}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
   <si>
     <t>hab_value</t>
   </si>
@@ -170,13 +170,13 @@
     <t>future_sampling_recommended</t>
   </si>
   <si>
-    <t>similar fish densities upstream and downstream</t>
-  </si>
-  <si>
-    <t>Fry observed upstream and downstream so suspect equivalent densities</t>
-  </si>
-  <si>
     <t>Deactivate</t>
+  </si>
+  <si>
+    <t>pscis_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fry observed upstream and downstream </t>
   </si>
 </sst>
 </file>
@@ -528,19 +528,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A10DE3F-E4A8-B34E-806F-E8347038A62A}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -548,412 +549,433 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>0</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>2</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>197555</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>675</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3">
+        <v>197555</v>
+      </c>
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>700</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4">
+        <v>197555</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>197555</v>
+      </c>
+      <c r="D5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6">
+        <v>197559</v>
+      </c>
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>980</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7">
+        <v>197559</v>
+      </c>
+      <c r="D7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8">
+        <v>197533</v>
+      </c>
+      <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>125</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>41</v>
       </c>
-      <c r="J8" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8">
+      <c r="K8" t="s">
+        <v>45</v>
+      </c>
+      <c r="L8">
         <v>0.125</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9">
+        <v>197533</v>
+      </c>
+      <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>23</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>24</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>725</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>26</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>650</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>25</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>43</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>170</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>25</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>27</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>28</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>29</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>400</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>41</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>28</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>30</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>28</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>31</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>700</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>10</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>40</v>
       </c>
-      <c r="J17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>28</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>32</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>100</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>28</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>28</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>35</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>36</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>740</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>10</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>40</v>
       </c>
-      <c r="J21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>35</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>37</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>255</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>28</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>38</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>730</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>40</v>
       </c>
-      <c r="J23" t="s">
-        <v>46</v>
-      </c>
-      <c r="L23" t="s">
+      <c r="K23" t="s">
+        <v>47</v>
+      </c>
+      <c r="M23" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>28</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>39</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>630</v>
       </c>
     </row>

</xml_diff>

<commit_message>
build phase 2 template, add summary tables, test table links
</commit_message>
<xml_diff>
--- a/data/habitat_confirmations_priorities.xlsx
+++ b/data/habitat_confirmations_priorities.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\OneDrive\New_Graph\Current\2020-025_cwf_elk\scripts\fish_passage_elk_2020_reporting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46A152F-750A-41EB-9C6C-5C013CD1F34C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A41F917-60A4-4A20-B78F-BF90FB56784F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{821C12C4-A1B8-974C-A56E-63CAEF8E23F0}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
   <si>
     <t>hab_value</t>
   </si>
@@ -44,9 +44,6 @@
     <t>comments</t>
   </si>
   <si>
-    <t>length_of_new_habitat</t>
-  </si>
-  <si>
     <t>gazetted_names</t>
   </si>
   <si>
@@ -74,33 +71,9 @@
     <t>Unnamed Tributary to Elk River</t>
   </si>
   <si>
-    <t>4605732_us</t>
-  </si>
-  <si>
-    <t>4605732_ds</t>
-  </si>
-  <si>
-    <t>4605732_us_ef</t>
-  </si>
-  <si>
-    <t>4605732_ds_ef</t>
-  </si>
-  <si>
     <t>Brule Creek</t>
   </si>
   <si>
-    <t>4600070_us</t>
-  </si>
-  <si>
-    <t>4600070_us_ef</t>
-  </si>
-  <si>
-    <t>4600183_us</t>
-  </si>
-  <si>
-    <t>4600183_ds</t>
-  </si>
-  <si>
     <t>Unnamed Tributary to Grave Creek</t>
   </si>
   <si>
@@ -155,9 +128,6 @@
     <t>62516_ds</t>
   </si>
   <si>
-    <t>mod</t>
-  </si>
-  <si>
     <t>high</t>
   </si>
   <si>
@@ -173,10 +143,55 @@
     <t>Deactivate</t>
   </si>
   <si>
-    <t>pscis_id</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fry observed upstream and downstream </t>
+  </si>
+  <si>
+    <t>197555_us</t>
+  </si>
+  <si>
+    <t>197555_ds</t>
+  </si>
+  <si>
+    <t>197559_us</t>
+  </si>
+  <si>
+    <t>197533_us</t>
+  </si>
+  <si>
+    <t>197533_ds</t>
+  </si>
+  <si>
+    <t>197559_us_ef</t>
+  </si>
+  <si>
+    <t>197555_ds_ef</t>
+  </si>
+  <si>
+    <t>197555_us_ef</t>
+  </si>
+  <si>
+    <t>recommendation</t>
+  </si>
+  <si>
+    <t>upstream_habitat_length_m</t>
+  </si>
+  <si>
+    <t>habitat_value_rationale</t>
+  </si>
+  <si>
+    <t>species_codes</t>
+  </si>
+  <si>
+    <t>BT</t>
+  </si>
+  <si>
+    <t>BT, WCT</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>moderate</t>
   </si>
 </sst>
 </file>
@@ -192,12 +207,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -212,8 +233,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,34 +550,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A10DE3F-E4A8-B34E-806F-E8347038A62A}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.5" customWidth="1"/>
-    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="4" max="4" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="9" max="9" width="19.875" customWidth="1"/>
+    <col min="14" max="14" width="14.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>8</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>
@@ -564,10 +587,10 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I1" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="J1" t="s">
         <v>1</v>
@@ -576,406 +599,400 @@
         <v>2</v>
       </c>
       <c r="L1" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="N1" t="s">
+        <v>48</v>
+      </c>
+      <c r="O1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2">
-        <v>197555</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2">
         <v>675</v>
       </c>
-      <c r="F2" t="s">
-        <v>10</v>
+      <c r="E2" t="s">
+        <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="N2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3">
-        <v>197555</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3">
         <v>700</v>
       </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4">
-        <v>197555</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5">
-        <v>197555</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>197559</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6">
         <v>980</v>
       </c>
-      <c r="F6" t="s">
-        <v>10</v>
+      <c r="E6" t="s">
+        <v>9</v>
       </c>
       <c r="J6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="N6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7">
-        <v>197559</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8">
-        <v>197533</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8">
         <v>125</v>
       </c>
       <c r="J8" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="K8" t="s">
-        <v>45</v>
-      </c>
-      <c r="L8">
+        <v>35</v>
+      </c>
+      <c r="M8">
         <v>0.125</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9">
-        <v>197533</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9">
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11">
         <v>725</v>
       </c>
       <c r="J11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12">
         <v>650</v>
       </c>
       <c r="J12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13">
         <v>170</v>
       </c>
       <c r="J13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15">
         <v>400</v>
       </c>
       <c r="J15" t="s">
-        <v>41</v>
-      </c>
-      <c r="M15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="O15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16">
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>700</v>
+      </c>
+      <c r="E17" t="s">
+        <v>9</v>
+      </c>
+      <c r="H17" t="s">
         <v>31</v>
       </c>
-      <c r="E17">
-        <v>700</v>
-      </c>
-      <c r="F17" t="s">
-        <v>10</v>
-      </c>
       <c r="J17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18">
         <v>100</v>
       </c>
-      <c r="F18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+      <c r="H18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20">
+      <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21">
         <v>740</v>
       </c>
-      <c r="F21" t="s">
-        <v>10</v>
+      <c r="E21" t="s">
+        <v>9</v>
       </c>
       <c r="J21" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
-      </c>
-      <c r="D22" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22">
+        <v>26</v>
+      </c>
+      <c r="C22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22">
         <v>255</v>
       </c>
-      <c r="F22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23">
+        <v>19</v>
+      </c>
+      <c r="C23" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23">
         <v>730</v>
       </c>
       <c r="J23" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="K23" t="s">
-        <v>47</v>
-      </c>
-      <c r="M23" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="O23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24">
         <v>630</v>
       </c>
     </row>

</xml_diff>